<commit_message>
Cleaning up waste from repo
</commit_message>
<xml_diff>
--- a/data/rf_params/AutonoMS_template.xlsx
+++ b/data/rf_params/AutonoMS_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chalmers-my.sharepoint.com/personal/danbru_chalmers_se/Documents/Desktop/GenExp/data/rf_params/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{C1FFB6D1-7540-FD4B-8FAA-58D1BC3914CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{429C1423-3407-024F-BF8F-59AB759E3181}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{C1FFB6D1-7540-FD4B-8FAA-58D1BC3914CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2987D43-7C90-2E4E-8D88-336BBD6BC02B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19940" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="samples" sheetId="1" r:id="rId1"/>
@@ -759,10 +759,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1148,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1397,16 +1393,16 @@
         <v>600</v>
       </c>
       <c r="C31">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="D31">
         <v>0</v>
       </c>
       <c r="E31">
-        <v>3000</v>
+        <v>7000</v>
       </c>
       <c r="F31">
-        <v>500</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>